<commit_message>
Auto-refresh chess stats 2026-08-06
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>77 (54.2%)</t>
+          <t>77 (53.5%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>62 (43.7%)</t>
+          <t>64 (44.4%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>37 (45.7%)</t>
+          <t>38 (46.3%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5 (6.2%)</t>
+          <t>5 (6.1%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>39 (48.1%)</t>
+          <t>39 (47.6%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15 (51.7%)</t>
+          <t>15 (50.0%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2 (6.9%)</t>
+          <t>2 (6.7%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>12 (41.4%)</t>
+          <t>13 (43.3%)</t>
         </is>
       </c>
     </row>
@@ -1067,21 +1067,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13 (48.1%)</t>
+          <t>14 (50.0%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2 (7.4%)</t>
+          <t>2 (7.1%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>12 (44.4%)</t>
+          <t>12 (42.9%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-07
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>77 (53.5%)</t>
+          <t>79 (53.0%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3 (2.1%)</t>
+          <t>5 (3.4%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>64 (44.4%)</t>
+          <t>65 (43.6%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>38 (46.3%)</t>
+          <t>38 (45.8%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5 (6.1%)</t>
+          <t>5 (6.0%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>39 (47.6%)</t>
+          <t>40 (48.2%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15 (50.0%)</t>
+          <t>15 (48.4%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2 (6.7%)</t>
+          <t>3 (9.7%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13 (43.3%)</t>
+          <t>13 (41.9%)</t>
         </is>
       </c>
     </row>
@@ -676,21 +676,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>9 (47.4%)</t>
+          <t>10 (50.0%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1 (5.3%)</t>
+          <t>1 (5.0%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>9 (47.4%)</t>
+          <t>9 (45.0%)</t>
         </is>
       </c>
     </row>
@@ -867,21 +867,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>73 (48.7%)</t>
+          <t>73 (48.3%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7 (4.7%)</t>
+          <t>7 (4.6%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>70 (46.7%)</t>
+          <t>71 (47.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-08
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>79 (53.0%)</t>
+          <t>80 (53.0%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (3.4%)</t>
+          <t>5 (3.3%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>65 (43.6%)</t>
+          <t>66 (43.7%)</t>
         </is>
       </c>
     </row>
@@ -501,11 +501,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>22 (46.8%)</t>
+          <t>23 (47.9%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>25 (53.2%)</t>
+          <t>25 (52.1%)</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -705,7 +705,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12 (66.7%)</t>
+          <t>11 (61.1%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -715,14 +715,14 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>5 (27.8%)</t>
+          <t>6 (33.3%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -730,42 +730,42 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>11 (61.1%)</t>
+          <t>9 (50.0%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1 (5.6%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>6 (33.3%)</t>
+          <t>9 (50.0%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>8 (50.0%)</t>
+          <t>12 (66.7%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (5.6%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>8 (50.0%)</t>
+          <t>5 (27.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-09
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>80 (53.0%)</t>
+          <t>81 (53.3%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>66 (43.7%)</t>
+          <t>66 (43.4%)</t>
         </is>
       </c>
     </row>
@@ -601,21 +601,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15 (65.2%)</t>
+          <t>16 (66.7%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (4.3%)</t>
+          <t>1 (4.2%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>7 (30.4%)</t>
+          <t>7 (29.2%)</t>
         </is>
       </c>
     </row>
@@ -626,21 +626,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10 (47.6%)</t>
+          <t>10 (45.5%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (4.8%)</t>
+          <t>1 (4.5%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>10 (47.6%)</t>
+          <t>11 (50.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-10
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>81 (53.3%)</t>
+          <t>81 (52.9%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>66 (43.4%)</t>
+          <t>67 (43.8%)</t>
         </is>
       </c>
     </row>
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>23 (47.9%)</t>
+          <t>23 (46.9%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (2.0%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>25 (52.1%)</t>
+          <t>25 (51.0%)</t>
         </is>
       </c>
     </row>
@@ -526,21 +526,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>27 (58.7%)</t>
+          <t>27 (57.4%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1 (2.2%)</t>
+          <t>1 (2.1%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>18 (39.1%)</t>
+          <t>19 (40.4%)</t>
         </is>
       </c>
     </row>
@@ -626,21 +626,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10 (45.5%)</t>
+          <t>11 (47.8%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (4.5%)</t>
+          <t>1 (4.3%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>11 (50.0%)</t>
+          <t>11 (47.8%)</t>
         </is>
       </c>
     </row>
@@ -697,32 +697,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11 (61.1%)</t>
+          <t>9 (47.4%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1 (5.6%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>6 (33.3%)</t>
+          <t>10 (52.6%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -730,17 +730,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>9 (50.0%)</t>
+          <t>11 (61.1%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (5.6%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>9 (50.0%)</t>
+          <t>6 (33.3%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-11
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>81 (52.9%)</t>
+          <t>82 (53.2%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (3.3%)</t>
+          <t>5 (3.2%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>67 (43.8%)</t>
+          <t>67 (43.5%)</t>
         </is>
       </c>
     </row>
@@ -501,11 +501,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>23 (46.9%)</t>
+          <t>24 (48.0%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>25 (51.0%)</t>
+          <t>25 (50.0%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15 (46.9%)</t>
+          <t>15 (45.5%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>4 (12.5%)</t>
+          <t>5 (15.2%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13 (40.6%)</t>
+          <t>13 (39.4%)</t>
         </is>
       </c>
     </row>
@@ -576,21 +576,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10 (34.5%)</t>
+          <t>10 (33.3%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2 (6.9%)</t>
+          <t>2 (6.7%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17 (58.6%)</t>
+          <t>18 (60.0%)</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -730,7 +730,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>11 (61.1%)</t>
+          <t>12 (66.7%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -740,14 +740,14 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>6 (33.3%)</t>
+          <t>5 (27.8%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -755,7 +755,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>12 (66.7%)</t>
+          <t>11 (61.1%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>5 (27.8%)</t>
+          <t>6 (33.3%)</t>
         </is>
       </c>
     </row>
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7 (43.8%)</t>
+          <t>7 (41.2%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -790,7 +790,32 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9 (56.2%)</t>
+          <t>10 (58.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>5 (33.3%)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2 (13.3%)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>8 (53.3%)</t>
         </is>
       </c>
     </row>
@@ -867,11 +892,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>73 (48.3%)</t>
+          <t>74 (48.7%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -881,7 +906,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>71 (47.0%)</t>
+          <t>71 (46.7%)</t>
         </is>
       </c>
     </row>
@@ -1142,21 +1167,21 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>9 (37.5%)</t>
+          <t>10 (40.0%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2 (8.3%)</t>
+          <t>2 (8.0%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13 (54.2%)</t>
+          <t>13 (52.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-12
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>82 (53.2%)</t>
+          <t>82 (52.9%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>67 (43.5%)</t>
+          <t>68 (43.9%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>39 (46.4%)</t>
+          <t>41 (47.7%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5 (6.0%)</t>
+          <t>5 (5.8%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>40 (47.6%)</t>
+          <t>40 (46.5%)</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Russian Federation</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -685,37 +685,37 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1 (5.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>9 (45.0%)</t>
+          <t>10 (50.0%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Russian Federation</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>9 (47.4%)</t>
+          <t>10 (50.0%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (5.0%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10 (52.6%)</t>
+          <t>9 (45.0%)</t>
         </is>
       </c>
     </row>
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7 (41.2%)</t>
+          <t>8 (44.4%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10 (58.8%)</t>
+          <t>10 (55.6%)</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1246,24 +1246,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14 (70.0%)</t>
+          <t>10 (50.0%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1 (5.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>5 (25.0%)</t>
+          <t>10 (50.0%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1276,27 +1276,27 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (5.0%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6 (30.0%)</t>
+          <t>5 (25.0%)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>10 (52.6%)</t>
+          <t>14 (70.0%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>9 (47.4%)</t>
+          <t>6 (30.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-13
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -526,11 +526,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>27 (57.4%)</t>
+          <t>28 (58.3%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>19 (40.4%)</t>
+          <t>19 (39.6%)</t>
         </is>
       </c>
     </row>
@@ -601,21 +601,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16 (66.7%)</t>
+          <t>17 (68.0%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (4.2%)</t>
+          <t>1 (4.0%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>7 (29.2%)</t>
+          <t>7 (28.0%)</t>
         </is>
       </c>
     </row>
@@ -722,32 +722,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12 (66.7%)</t>
+          <t>11 (57.9%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1 (5.6%)</t>
+          <t>1 (5.3%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>5 (27.8%)</t>
+          <t>7 (36.8%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -755,7 +755,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11 (61.1%)</t>
+          <t>12 (66.7%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>6 (33.3%)</t>
+          <t>5 (27.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-14
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>82 (52.9%)</t>
+          <t>82 (52.2%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>68 (43.9%)</t>
+          <t>70 (44.6%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>41 (47.7%)</t>
+          <t>42 (48.3%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5 (5.8%)</t>
+          <t>5 (5.7%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>40 (46.5%)</t>
+          <t>40 (46.0%)</t>
         </is>
       </c>
     </row>
@@ -651,11 +651,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8 (38.1%)</t>
+          <t>8 (36.4%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>13 (61.9%)</t>
+          <t>14 (63.6%)</t>
         </is>
       </c>
     </row>
@@ -892,11 +892,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>74 (48.7%)</t>
+          <t>75 (49.0%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>71 (46.7%)</t>
+          <t>71 (46.4%)</t>
         </is>
       </c>
     </row>
@@ -992,21 +992,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>18 (40.9%)</t>
+          <t>18 (40.0%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>7 (15.9%)</t>
+          <t>7 (15.6%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>19 (43.2%)</t>
+          <t>20 (44.4%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-15
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -497,7 +497,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -505,7 +505,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>24 (48.0%)</t>
+          <t>29 (58.0%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,32 +515,32 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>25 (50.0%)</t>
+          <t>20 (40.0%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>28 (58.3%)</t>
+          <t>24 (48.0%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1 (2.1%)</t>
+          <t>1 (2.0%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>19 (39.6%)</t>
+          <t>25 (50.0%)</t>
         </is>
       </c>
     </row>
@@ -601,21 +601,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17 (68.0%)</t>
+          <t>17 (65.4%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (4.0%)</t>
+          <t>1 (3.8%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>7 (28.0%)</t>
+          <t>8 (30.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-16
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>82 (52.2%)</t>
+          <t>84 (52.8%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (3.2%)</t>
+          <t>5 (3.1%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>70 (44.6%)</t>
+          <t>70 (44.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-21
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15 (45.5%)</t>
+          <t>16 (47.1%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5 (15.2%)</t>
+          <t>5 (14.7%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13 (39.4%)</t>
+          <t>13 (38.2%)</t>
         </is>
       </c>
     </row>
@@ -672,32 +672,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Russian Federation</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10 (50.0%)</t>
+          <t>10 (47.6%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (4.8%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>10 (50.0%)</t>
+          <t>10 (47.6%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Russian Federation</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -710,12 +710,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1 (5.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>9 (45.0%)</t>
+          <t>10 (50.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-22
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>16 (47.1%)</t>
+          <t>16 (45.7%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5 (14.7%)</t>
+          <t>6 (17.1%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13 (38.2%)</t>
+          <t>13 (37.1%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-24
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -626,21 +626,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11 (47.8%)</t>
+          <t>12 (50.0%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (4.3%)</t>
+          <t>1 (4.2%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>11 (47.8%)</t>
+          <t>11 (45.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-25
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -626,21 +626,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12 (50.0%)</t>
+          <t>12 (48.0%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (4.2%)</t>
+          <t>1 (4.0%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>11 (45.8%)</t>
+          <t>12 (48.0%)</t>
         </is>
       </c>
     </row>
@@ -726,21 +726,21 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>11 (57.9%)</t>
+          <t>11 (55.0%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1 (5.3%)</t>
+          <t>1 (5.0%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>7 (36.8%)</t>
+          <t>8 (40.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-26
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>84 (52.8%)</t>
+          <t>86 (53.4%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>70 (44.0%)</t>
+          <t>70 (43.5%)</t>
         </is>
       </c>
     </row>
@@ -626,21 +626,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12 (48.0%)</t>
+          <t>12 (46.2%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (4.0%)</t>
+          <t>2 (7.7%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>12 (48.0%)</t>
+          <t>12 (46.2%)</t>
         </is>
       </c>
     </row>
@@ -867,11 +867,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>99 (50.5%)</t>
+          <t>100 (50.8%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>89 (45.4%)</t>
+          <t>89 (45.2%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-27
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>29 (58.0%)</t>
+          <t>31 (59.6%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1 (2.0%)</t>
+          <t>1 (1.9%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20 (40.0%)</t>
+          <t>20 (38.5%)</t>
         </is>
       </c>
     </row>
@@ -526,11 +526,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>24 (48.0%)</t>
+          <t>25 (49.0%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>25 (50.0%)</t>
+          <t>25 (49.0%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>16 (45.7%)</t>
+          <t>17 (47.2%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (17.1%)</t>
+          <t>6 (16.7%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13 (37.1%)</t>
+          <t>13 (36.1%)</t>
         </is>
       </c>
     </row>
@@ -676,53 +676,53 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10 (47.6%)</t>
+          <t>11 (50.0%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1 (4.8%)</t>
+          <t>1 (4.5%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>10 (47.6%)</t>
+          <t>10 (45.5%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10 (50.0%)</t>
+          <t>12 (57.1%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (4.8%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10 (50.0%)</t>
+          <t>8 (38.1%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -730,17 +730,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>11 (55.0%)</t>
+          <t>10 (50.0%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1 (5.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>8 (40.0%)</t>
+          <t>10 (50.0%)</t>
         </is>
       </c>
     </row>
@@ -801,21 +801,21 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5 (33.3%)</t>
+          <t>6 (37.5%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2 (13.3%)</t>
+          <t>2 (12.5%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>8 (53.3%)</t>
+          <t>8 (50.0%)</t>
         </is>
       </c>
     </row>
@@ -917,21 +917,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>27 (40.3%)</t>
+          <t>28 (41.2%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5 (7.5%)</t>
+          <t>5 (7.4%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>35 (52.2%)</t>
+          <t>35 (51.5%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-28
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -747,32 +747,32 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>12 (66.7%)</t>
+          <t>8 (42.1%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1 (5.6%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>5 (27.8%)</t>
+          <t>11 (57.9%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -780,17 +780,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>8 (44.4%)</t>
+          <t>12 (66.7%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (5.6%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10 (55.6%)</t>
+          <t>5 (27.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-29
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -651,11 +651,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8 (36.4%)</t>
+          <t>9 (39.1%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14 (63.6%)</t>
+          <t>14 (60.9%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-30
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>86 (53.4%)</t>
+          <t>87 (53.7%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>70 (43.5%)</t>
+          <t>70 (43.2%)</t>
         </is>
       </c>
     </row>
@@ -501,11 +501,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>31 (59.6%)</t>
+          <t>31 (58.5%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20 (38.5%)</t>
+          <t>21 (39.6%)</t>
         </is>
       </c>
     </row>
@@ -597,32 +597,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17 (65.4%)</t>
+          <t>12 (44.4%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (3.8%)</t>
+          <t>2 (7.4%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>8 (30.8%)</t>
+          <t>13 (48.1%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -630,17 +630,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12 (46.2%)</t>
+          <t>17 (65.4%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2 (7.7%)</t>
+          <t>1 (3.8%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>12 (46.2%)</t>
+          <t>8 (30.8%)</t>
         </is>
       </c>
     </row>
@@ -801,21 +801,21 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>6 (37.5%)</t>
+          <t>7 (41.2%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2 (12.5%)</t>
+          <t>2 (11.8%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>8 (50.0%)</t>
+          <t>8 (47.1%)</t>
         </is>
       </c>
     </row>
@@ -867,21 +867,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100 (50.8%)</t>
+          <t>100 (50.5%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8 (4.1%)</t>
+          <t>8 (4.0%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>89 (45.2%)</t>
+          <t>90 (45.5%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-08-31
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>87 (53.7%)</t>
+          <t>87 (53.4%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>70 (43.2%)</t>
+          <t>71 (43.6%)</t>
         </is>
       </c>
     </row>
@@ -476,11 +476,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>42 (48.3%)</t>
+          <t>42 (47.7%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>40 (46.0%)</t>
+          <t>41 (46.6%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17 (47.2%)</t>
+          <t>18 (48.6%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (16.7%)</t>
+          <t>6 (16.2%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13 (36.1%)</t>
+          <t>13 (35.1%)</t>
         </is>
       </c>
     </row>
@@ -651,11 +651,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9 (39.1%)</t>
+          <t>10 (41.7%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14 (60.9%)</t>
+          <t>14 (58.3%)</t>
         </is>
       </c>
     </row>
@@ -892,21 +892,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>75 (49.0%)</t>
+          <t>75 (48.7%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7 (4.6%)</t>
+          <t>7 (4.5%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>71 (46.4%)</t>
+          <t>72 (46.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-01
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18 (48.6%)</t>
+          <t>18 (47.4%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (16.2%)</t>
+          <t>6 (15.8%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13 (35.1%)</t>
+          <t>14 (36.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-02
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>87 (53.4%)</t>
+          <t>88 (53.7%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (3.1%)</t>
+          <t>5 (3.0%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>71 (43.6%)</t>
+          <t>71 (43.3%)</t>
         </is>
       </c>
     </row>
@@ -526,21 +526,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>25 (49.0%)</t>
+          <t>25 (48.1%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1 (2.0%)</t>
+          <t>1 (1.9%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>25 (49.0%)</t>
+          <t>26 (50.0%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18 (47.4%)</t>
+          <t>18 (46.2%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (15.8%)</t>
+          <t>6 (15.4%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14 (36.8%)</t>
+          <t>15 (38.5%)</t>
         </is>
       </c>
     </row>
@@ -672,50 +672,50 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Russian Federation</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11 (50.0%)</t>
+          <t>12 (52.2%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1 (4.5%)</t>
+          <t>1 (4.3%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>10 (45.5%)</t>
+          <t>10 (43.5%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Russian Federation</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12 (57.1%)</t>
+          <t>11 (50.0%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1 (4.8%)</t>
+          <t>1 (4.5%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>8 (38.1%)</t>
+          <t>10 (45.5%)</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -780,42 +780,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>12 (66.7%)</t>
+          <t>7 (38.9%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1 (5.6%)</t>
+          <t>2 (11.1%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>5 (27.8%)</t>
+          <t>9 (50.0%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>7 (41.2%)</t>
+          <t>12 (66.7%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2 (11.8%)</t>
+          <t>1 (5.6%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>8 (47.1%)</t>
+          <t>5 (27.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-03
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -501,11 +501,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>31 (58.5%)</t>
+          <t>31 (57.4%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>21 (39.6%)</t>
+          <t>22 (40.7%)</t>
         </is>
       </c>
     </row>
@@ -676,21 +676,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12 (52.2%)</t>
+          <t>12 (50.0%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1 (4.3%)</t>
+          <t>1 (4.2%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>10 (43.5%)</t>
+          <t>11 (45.8%)</t>
         </is>
       </c>
     </row>
@@ -701,21 +701,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11 (50.0%)</t>
+          <t>12 (52.2%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1 (4.5%)</t>
+          <t>1 (4.3%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10 (45.5%)</t>
+          <t>10 (43.5%)</t>
         </is>
       </c>
     </row>
@@ -726,11 +726,11 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10 (50.0%)</t>
+          <t>10 (47.6%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>10 (50.0%)</t>
+          <t>11 (52.4%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-04
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>88 (53.7%)</t>
+          <t>89 (53.3%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>71 (43.3%)</t>
+          <t>73 (43.7%)</t>
         </is>
       </c>
     </row>
@@ -601,21 +601,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12 (44.4%)</t>
+          <t>12 (41.4%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2 (7.4%)</t>
+          <t>2 (6.9%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>13 (48.1%)</t>
+          <t>15 (51.7%)</t>
         </is>
       </c>
     </row>
@@ -701,21 +701,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12 (52.2%)</t>
+          <t>13 (54.2%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1 (4.3%)</t>
+          <t>1 (4.2%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10 (43.5%)</t>
+          <t>10 (41.7%)</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -755,49 +755,49 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>8 (42.1%)</t>
+          <t>12 (63.2%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (5.3%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11 (57.9%)</t>
+          <t>6 (31.6%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7 (38.9%)</t>
+          <t>8 (42.1%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2 (11.1%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>9 (50.0%)</t>
+          <t>11 (57.9%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -805,17 +805,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>12 (66.7%)</t>
+          <t>7 (38.9%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1 (5.6%)</t>
+          <t>2 (11.1%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>5 (27.8%)</t>
+          <t>9 (50.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-05
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>89 (53.3%)</t>
+          <t>89 (53.0%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>73 (43.7%)</t>
+          <t>74 (44.0%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>42 (47.7%)</t>
+          <t>43 (47.8%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5 (5.7%)</t>
+          <t>5 (5.6%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>41 (46.6%)</t>
+          <t>42 (46.7%)</t>
         </is>
       </c>
     </row>
@@ -647,32 +647,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10 (41.7%)</t>
+          <t>12 (48.0%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (4.0%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14 (58.3%)</t>
+          <t>12 (48.0%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -680,17 +680,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12 (50.0%)</t>
+          <t>10 (41.7%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1 (4.2%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>11 (45.8%)</t>
+          <t>14 (58.3%)</t>
         </is>
       </c>
     </row>

</xml_diff>